<commit_message>
feat(catalog): 異體字加 4 格 Unicode 悉曇（__i 𑗘／_i 𑗙／_ii 𑗚／__u 𑗛）＋ scripts/build-catalog.py
- BonjiInput.xlsx 的 variant sheet 加 4 列（group siddham，排在 Mojikyo 3 列之前）〔owner 2026-10-08〕
- 補上 xlsx → catalog.json 的產生器（DESIGN §7.2 一直描述、但不在 repo 裡）；補上時先證明對當時的 xlsx
  逐位元組重產出既有 catalog.json，才去改 xlsx（xlsx 只動 sheet3.xml，其餘 zip 成員逐位元組相同）
- 輔助輸入預設群 278 → 282、合計 625 → 629；新的 4 格有記法、可插入，Mojikyo 3 格維持不可插入
- ⚠️ __u 不是引擎的記法：轉換層把 _u 定義成替代母音符號，__u 轉得出 𑗛 是它的副作用（DESIGN §7.4）

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/apps/bonji/data/BonjiInput.xlsx
+++ b/public/apps/bonji/data/BonjiInput.xlsx
@@ -3646,7 +3646,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4941B66-DEBD-407D-B4E4-003448730531}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="18" customWidth="1"/>
@@ -3677,13 +3677,17 @@
         <v>202</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>203</v>
+        <v>6</v>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>__i</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>𑗘</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -3694,13 +3698,17 @@
         <v>202</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>204</v>
+        <v>6</v>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>_i</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>𑗙</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -3711,12 +3719,88 @@
         <v>202</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>_ii</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>𑗚</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="12">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>__u</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>𑗛</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="12">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E6" s="11" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="12">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="12">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>205</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(catalog): 接續加 6 格 CBETA 字形（uniSiddham：.t 盄／.th 眈／.dh 眄／th 盷／n 矧／lla;m 祋）
- BonjiInput.xlsx 的接續表加 6 列，各自緊接在同音的 Unicode 那一列之後（祋 接在 h 之後）〔owner 2026-10-09〕
  只動 sheet6.xml；catalog.json 差異正好是接續 35 → 41、其餘逐一不變
- 盷 原清單 input 寫 .th，與 after 欄 𑖞𑖿 及 db_siddham（齒音 tha）不符——owner 裁定 th
- 輔助輸入預設群 282 → 288、合計 629 → 635；缺字型標記格數實數 DOM：catalog 頁 151 → 157、轉換頁 497 → 504
  （497 在此前就已落後 1：Mojikyo 群 2026-09-01 補 空 而文件沒跟上）

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/apps/bonji/data/BonjiInput.xlsx
+++ b/public/apps/bonji/data/BonjiInput.xlsx
@@ -4687,7 +4687,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF7BF155-14E5-441B-A4E8-13500DF285AE}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="17.83203125" customWidth="1"/>
@@ -4898,20 +4898,24 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="18">
+      <c r="A13" s="12">
         <v>12</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>276</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>277</v>
+      <c r="C13" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>.t</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>盄</t>
+        </is>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -4925,27 +4929,31 @@
         <v>6</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="18">
+      <c r="A15" s="12">
         <v>14</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="C15" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>280</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>281</v>
+      <c r="C15" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>.th</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>眈</t>
+        </is>
       </c>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -4959,10 +4967,10 @@
         <v>6</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -4972,31 +4980,35 @@
       <c r="B17" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>44</v>
+      <c r="C17" s="17" t="s">
+        <v>6</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="18">
+      <c r="A18" s="12">
         <v>17</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="C18" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>285</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>286</v>
+      <c r="C18" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>.dh</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>眄</t>
+        </is>
       </c>
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5010,10 +5022,10 @@
         <v>6</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5023,14 +5035,14 @@
       <c r="B20" s="17" t="s">
         <v>253</v>
       </c>
-      <c r="C20" s="17" t="s">
-        <v>6</v>
+      <c r="C20" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5044,10 +5056,10 @@
         <v>6</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5061,27 +5073,31 @@
         <v>6</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="18">
+      <c r="A23" s="12">
         <v>22</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="C23" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>295</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>296</v>
+      <c r="C23" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>th</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>盷</t>
+        </is>
       </c>
     </row>
     <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5095,10 +5111,10 @@
         <v>6</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5112,10 +5128,10 @@
         <v>6</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5129,27 +5145,31 @@
         <v>6</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="18">
+      <c r="A27" s="12">
         <v>26</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="C27" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>303</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>304</v>
+      <c r="C27" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>矧</t>
+        </is>
       </c>
     </row>
     <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5163,10 +5183,10 @@
         <v>6</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5180,10 +5200,10 @@
         <v>6</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5197,10 +5217,10 @@
         <v>6</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5214,10 +5234,10 @@
         <v>6</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5231,10 +5251,10 @@
         <v>6</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5248,10 +5268,10 @@
         <v>6</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5265,10 +5285,10 @@
         <v>6</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5282,10 +5302,10 @@
         <v>6</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -5299,9 +5319,115 @@
         <v>6</v>
       </c>
       <c r="D36" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="18">
+        <v>36</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="18">
+        <v>37</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="18">
+        <v>38</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40" s="18">
+        <v>39</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C40" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="12">
+        <v>40</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>lla;m</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>祋</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="18">
+        <v>41</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="E36" s="17" t="s">
+      <c r="E42" s="17" t="s">
         <v>322</v>
       </c>
     </row>

</xml_diff>